<commit_message>
feat: implement power bi fabric automation deployment pipeline with workspace and report management tools
</commit_message>
<xml_diff>
--- a/data/refresh_schedule.xlsx
+++ b/data/refresh_schedule.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B22"/>
+  <dimension ref="A1:B23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -479,7 +479,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Ademar</t>
+          <t>Ademar Cruz</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -515,7 +515,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Cleide</t>
+          <t>Cleide Lima</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -527,7 +527,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Edvaldo</t>
+          <t>Edvaldo Correa</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -563,7 +563,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Gilmara</t>
+          <t>Gilmara Dantas</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -599,7 +599,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Monique</t>
+          <t>Monique Bendahan</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -635,7 +635,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Silvana</t>
+          <t>Silvana Souza</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -675,6 +675,18 @@
         </is>
       </c>
       <c r="B22" t="inlineStr">
+        <is>
+          <t>08:00,18:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Superintendência</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
         <is>
           <t>08:00,18:00</t>
         </is>

</xml_diff>